<commit_message>
1058517: Added Spreadsheet Version History code in Python
</commit_message>
<xml_diff>
--- a/server/python/Files/Data/Sample.xlsx
+++ b/server/python/Files/Data/Sample.xlsx
@@ -8,133 +8,78 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Master\2026\Oct\Presale\PythonNew\Spreadsheet-Version-History\server\python\Files\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCC7E6EB-31BD-4139-AE08-D6326C92D7C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EF0A484-E755-49D7-8F6B-1BE75FEB1FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Property Information" sheetId="1" r:id="rId1"/>
+    <sheet name="Price Details" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
-  <si>
-    <t>Property ID</t>
-  </si>
-  <si>
-    <t>Property Name</t>
-  </si>
-  <si>
-    <t>Property Type</t>
-  </si>
-  <si>
-    <t>Address</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>State</t>
-  </si>
-  <si>
-    <t>Zip Code</t>
-  </si>
-  <si>
-    <t>Year Built</t>
-  </si>
-  <si>
-    <t>Building Class</t>
-  </si>
-  <si>
-    <t>Gross Building Area (Sq Ft)</t>
-  </si>
-  <si>
-    <t>Net Rentable Area (Sq Ft)</t>
-  </si>
-  <si>
-    <t>Land Area (Acres)</t>
-  </si>
-  <si>
-    <t>Number of Floors</t>
-  </si>
-  <si>
-    <t>Total Rental Units</t>
-  </si>
-  <si>
-    <t>Property Manager</t>
-  </si>
-  <si>
-    <t>Owner Name</t>
-  </si>
-  <si>
-    <t>Appraisal Date</t>
-  </si>
-  <si>
-    <t>Market Cap Rate</t>
-  </si>
-  <si>
-    <t>Average Annual Operating Expense</t>
-  </si>
-  <si>
-    <t>Average Annual Maintenance Expense</t>
-  </si>
-  <si>
-    <t>Property Condition</t>
-  </si>
-  <si>
-    <t>PROP-001</t>
-  </si>
-  <si>
-    <t>Sunset Towers</t>
-  </si>
-  <si>
-    <t>Commercial Office Building</t>
-  </si>
-  <si>
-    <t>125 Market Street</t>
-  </si>
-  <si>
-    <t>Chicago</t>
-  </si>
-  <si>
-    <t>IL</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Michael Johnson</t>
-  </si>
-  <si>
-    <t>Sunset Holdings LLC</t>
-  </si>
-  <si>
-    <t>Excellent</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+  <si>
+    <t>Item Name</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Time</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Discount</t>
+  </si>
+  <si>
+    <t>Profit</t>
+  </si>
+  <si>
+    <t>Casual Shoes</t>
+  </si>
+  <si>
+    <t>Sports Shoes</t>
+  </si>
+  <si>
+    <t>Formal Shoes</t>
+  </si>
+  <si>
+    <t>Sandals &amp; Floaters</t>
+  </si>
+  <si>
+    <t>Flip- Flops &amp; Slippers</t>
+  </si>
+  <si>
+    <t>Sneakers</t>
+  </si>
+  <si>
+    <t>Running Shoes</t>
+  </si>
+  <si>
+    <t>Loafers</t>
+  </si>
+  <si>
+    <t>Cricket Shoes</t>
+  </si>
+  <si>
+    <t>T-Shirts</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
-  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -147,22 +92,16 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E78"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -174,34 +113,26 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="7">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
-      <protection locked="0"/>
+  </cellStyleXfs>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="19" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
-      <protection locked="0"/>
-    </xf>
-  </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="7">
-    <cellStyle name="Appraisal SummaryLockedColumnStyle" xfId="5" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="Appraisal SummaryUnLockedColumnStyle" xfId="6" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Property InformationLockedColumnStyle" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="Property InformationUnLockedColumnStyle" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="Rent Roll DataLockedColumnStyle" xfId="3" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="Rent Roll DataUnLockedColumnStyle" xfId="4" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
+    <cellStyle name="Sheet1LockedColumnStyle" xfId="1" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Sheet1UnLockedColumnStyle" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0"/>
@@ -513,159 +444,298 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U2"/>
-  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.5546875" customWidth="1"/>
-    <col min="2" max="2" width="13.88671875" customWidth="1"/>
-    <col min="3" max="3" width="23.21875" customWidth="1"/>
-    <col min="4" max="4" width="15.6640625" customWidth="1"/>
-    <col min="5" max="5" width="7.44140625" customWidth="1"/>
-    <col min="6" max="6" width="5.21875" customWidth="1"/>
-    <col min="7" max="7" width="8.21875" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" customWidth="1"/>
-    <col min="10" max="10" width="23.21875" customWidth="1"/>
-    <col min="11" max="11" width="22.44140625" customWidth="1"/>
-    <col min="12" max="12" width="15.88671875" customWidth="1"/>
-    <col min="13" max="13" width="15.6640625" customWidth="1"/>
-    <col min="14" max="14" width="15.88671875" customWidth="1"/>
-    <col min="15" max="15" width="16.44140625" customWidth="1"/>
-    <col min="16" max="16" width="17.21875" customWidth="1"/>
-    <col min="17" max="17" width="13.21875" customWidth="1"/>
-    <col min="18" max="18" width="15.109375" customWidth="1"/>
-    <col min="19" max="19" width="31" customWidth="1"/>
-    <col min="20" max="20" width="33.88671875" customWidth="1"/>
-    <col min="21" max="21" width="17.21875" customWidth="1"/>
+    <col min="1" max="1" width="18.5546875" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="B2" s="1">
+        <v>41684</v>
+      </c>
+      <c r="C2" s="2">
+        <v>0.48231481481481497</v>
+      </c>
+      <c r="D2">
+        <v>10</v>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+      <c r="F2">
+        <v>200</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="B3" s="1">
+        <v>41801</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.247592592592593</v>
+      </c>
+      <c r="D3">
+        <v>20</v>
+      </c>
+      <c r="E3">
+        <v>30</v>
+      </c>
+      <c r="F3">
+        <v>600</v>
+      </c>
+      <c r="G3">
+        <v>5</v>
+      </c>
+      <c r="H3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="B4" s="1">
+        <v>41847</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.14773148148148099</v>
+      </c>
+      <c r="D4">
+        <v>20</v>
+      </c>
+      <c r="E4">
+        <v>15</v>
+      </c>
+      <c r="F4">
+        <v>300</v>
+      </c>
+      <c r="G4">
+        <v>7</v>
+      </c>
+      <c r="H4">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="B5" s="1">
+        <v>41964</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.26659722222222199</v>
+      </c>
+      <c r="D5">
+        <v>15</v>
+      </c>
+      <c r="E5">
+        <v>20</v>
+      </c>
+      <c r="F5">
+        <v>300</v>
+      </c>
+      <c r="G5">
+        <v>11</v>
+      </c>
+      <c r="H5">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="B6" s="1">
+        <v>41813</v>
+      </c>
+      <c r="C6" s="2">
+        <v>3.0543981481481498E-2</v>
+      </c>
+      <c r="D6">
+        <v>30</v>
+      </c>
+      <c r="E6">
+        <v>10</v>
+      </c>
+      <c r="F6">
+        <v>300</v>
+      </c>
+      <c r="G6">
+        <v>10</v>
+      </c>
+      <c r="H6">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="B7" s="1">
+        <v>41842</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.455474537037037</v>
+      </c>
+      <c r="D7">
+        <v>40</v>
+      </c>
+      <c r="E7">
+        <v>20</v>
+      </c>
+      <c r="F7">
+        <v>800</v>
+      </c>
+      <c r="G7">
+        <v>13</v>
+      </c>
+      <c r="H7">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="B8" s="1">
+        <v>41674</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0.15594907407407399</v>
+      </c>
+      <c r="D8">
+        <v>20</v>
+      </c>
+      <c r="E8">
+        <v>10</v>
+      </c>
+      <c r="F8">
+        <v>200</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+      <c r="H8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="B9" s="1">
+        <v>41973</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.13393518518518499</v>
+      </c>
+      <c r="D9">
+        <v>31</v>
+      </c>
+      <c r="E9">
+        <v>10</v>
+      </c>
+      <c r="F9">
+        <v>310</v>
+      </c>
+      <c r="G9">
+        <v>6</v>
+      </c>
+      <c r="H9">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="B10" s="1">
+        <v>41829</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0.480717592592593</v>
+      </c>
+      <c r="D10">
+        <v>41</v>
+      </c>
+      <c r="E10">
+        <v>30</v>
+      </c>
+      <c r="F10">
+        <v>1210</v>
+      </c>
+      <c r="G10">
+        <v>12</v>
+      </c>
+      <c r="H10">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" t="s">
-        <v>26</v>
-      </c>
-      <c r="G2">
-        <v>60601</v>
-      </c>
-      <c r="H2">
-        <v>2015</v>
-      </c>
-      <c r="I2" t="s">
-        <v>27</v>
-      </c>
-      <c r="J2">
-        <v>120000</v>
-      </c>
-      <c r="K2">
-        <v>100000</v>
-      </c>
-      <c r="L2">
-        <v>2.5</v>
-      </c>
-      <c r="M2">
-        <v>15</v>
-      </c>
-      <c r="N2">
+      <c r="B11" s="1">
+        <v>41943</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1.2037037037037001E-3</v>
+      </c>
+      <c r="D11">
         <v>50</v>
       </c>
-      <c r="O2" t="s">
-        <v>28</v>
-      </c>
-      <c r="P2" t="s">
-        <v>29</v>
-      </c>
-      <c r="Q2">
-        <v>46301</v>
-      </c>
-      <c r="R2">
-        <v>6.5000000000000002E-2</v>
-      </c>
-      <c r="S2" s="2">
-        <v>450000</v>
-      </c>
-      <c r="T2" s="2">
-        <v>120000</v>
-      </c>
-      <c r="U2" t="s">
-        <v>30</v>
+      <c r="E11">
+        <v>10</v>
+      </c>
+      <c r="F11">
+        <v>500</v>
+      </c>
+      <c r="G11">
+        <v>9</v>
+      </c>
+      <c r="H11">
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>